<commit_message>
Fix Package 18 typo
</commit_message>
<xml_diff>
--- a/curation/package18/R18_BC_DSS_BrCa_TAUG_2.xlsx
+++ b/curation/package18/R18_BC_DSS_BrCa_TAUG_2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Linda\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_github\cdisc-org\COSMoS\curation\package18\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801E0AAC-F3D5-4645-B306-DEF33474D364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB14E129-B708-4303-A984-4AB36B068FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13866" xr2:uid="{9C2B54C0-060B-496F-B408-7D0F2041239C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9C2B54C0-060B-496F-B408-7D0F2041239C}"/>
   </bookViews>
   <sheets>
     <sheet name="BC_BrCa" sheetId="1" r:id="rId1"/>
@@ -502,9 +502,6 @@
     <t>A technique for measuring the gamma radiation produced by collisions of electrons and positrons (anti-electrons) within living tissue. In positron emission tomography (PET), a subject is given a dose of a positron-emitting radionuclide attached to a metabolically active substance (for example, 2-fluoro-2-deoxy-D-glucose (FDG), which is similar to a naturally occurring sugar, glucose, with the addition of a radioactive fluorine atom). When living tissue containing the positron emitter is bombarded by electrons, gamma radiation produced by collisions of electrons and positrons is detected by a scanner, revealing in fine detail the tissue location of the metabolically-active substance administered.</t>
   </si>
   <si>
-    <t>Diagnostic Imaging;Medical Imaging;Tomagraphy</t>
-  </si>
-  <si>
     <t>PET SCAN</t>
   </si>
   <si>
@@ -620,13 +617,16 @@
   </si>
   <si>
     <t>CTSCANPELVIS</t>
+  </si>
+  <si>
+    <t>Diagnostic Imaging;Medical Imaging;Tomography</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1138,20 +1138,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02DBC567-A798-4813-83E1-012FB631D130}">
   <dimension ref="A1:R42"/>
-  <sheetFormatPr defaultRowHeight="14.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="30.29296875" customWidth="1"/>
-    <col min="6" max="6" width="33.1171875" customWidth="1"/>
-    <col min="7" max="7" width="24.87890625" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" customWidth="1"/>
+    <col min="6" max="6" width="33.140625" customWidth="1"/>
+    <col min="7" max="7" width="24.85546875" customWidth="1"/>
     <col min="9" max="9" width="45" customWidth="1"/>
     <col min="10" max="12" width="9" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="11.41015625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="32.703125" customWidth="1"/>
-    <col min="17" max="17" width="42.29296875" customWidth="1"/>
-    <col min="18" max="18" width="17.703125" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="32.7109375" customWidth="1"/>
+    <col min="17" max="17" width="42.28515625" customWidth="1"/>
+    <col min="18" max="18" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="3" customFormat="1" ht="14.1" customHeight="1">
+    <row r="1" spans="1:18" s="3" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" s="15" customFormat="1">
+    <row r="2" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>31</v>
       </c>
@@ -1215,10 +1215,10 @@
         <v>148</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E2" s="13"/>
       <c r="F2" s="12" t="s">
@@ -1238,7 +1238,7 @@
       <c r="P2" s="11"/>
       <c r="Q2" s="12"/>
     </row>
-    <row r="3" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="3" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>31</v>
       </c>
@@ -1252,10 +1252,10 @@
         <v>146</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>150</v>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="Q3" s="12"/>
     </row>
-    <row r="4" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="4" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>31</v>
       </c>
@@ -1297,10 +1297,10 @@
         <v>146</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G4" s="11" t="s">
         <v>150</v>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="Q4" s="12"/>
     </row>
-    <row r="5" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="5" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>31</v>
       </c>
@@ -1342,10 +1342,10 @@
         <v>146</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>150</v>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="Q5" s="12"/>
     </row>
-    <row r="6" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="6" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>31</v>
       </c>
@@ -1387,10 +1387,10 @@
         <v>146</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>150</v>
@@ -1418,7 +1418,7 @@
       </c>
       <c r="Q6" s="12"/>
     </row>
-    <row r="7" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="7" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
@@ -1432,10 +1432,10 @@
         <v>146</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>150</v>
@@ -1465,7 +1465,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="8" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>31</v>
       </c>
@@ -1479,10 +1479,10 @@
         <v>146</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>150</v>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="Q8" s="12"/>
     </row>
-    <row r="9" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="9" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>31</v>
       </c>
@@ -1524,10 +1524,10 @@
         <v>146</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>150</v>
@@ -1557,7 +1557,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="10" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="10" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>31</v>
       </c>
@@ -1571,10 +1571,10 @@
         <v>146</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>150</v>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="Q10" s="12"/>
     </row>
-    <row r="11" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="11" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>31</v>
       </c>
@@ -1616,10 +1616,10 @@
         <v>146</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>150</v>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="Q11" s="12"/>
     </row>
-    <row r="12" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="12" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>31</v>
       </c>
@@ -1661,10 +1661,10 @@
         <v>146</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>150</v>
@@ -1694,7 +1694,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="13" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>31</v>
       </c>
@@ -1708,10 +1708,10 @@
         <v>140</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>143</v>
@@ -1739,7 +1739,7 @@
       </c>
       <c r="Q13" s="12"/>
     </row>
-    <row r="14" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="14" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>31</v>
       </c>
@@ -1753,10 +1753,10 @@
         <v>140</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G14" s="11" t="s">
         <v>143</v>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="Q14" s="12"/>
     </row>
-    <row r="15" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="15" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>31</v>
       </c>
@@ -1798,10 +1798,10 @@
         <v>140</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G15" s="11" t="s">
         <v>143</v>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="Q15" s="12"/>
     </row>
-    <row r="16" spans="1:18" s="15" customFormat="1" ht="28.7">
+    <row r="16" spans="1:18" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>31</v>
       </c>
@@ -1843,10 +1843,10 @@
         <v>140</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G16" s="11" t="s">
         <v>143</v>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="Q16" s="12"/>
     </row>
-    <row r="17" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="17" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>31</v>
       </c>
@@ -1888,10 +1888,10 @@
         <v>140</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G17" s="11" t="s">
         <v>143</v>
@@ -1921,7 +1921,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="18" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>31</v>
       </c>
@@ -1935,10 +1935,10 @@
         <v>140</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G18" s="11" t="s">
         <v>143</v>
@@ -1968,7 +1968,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="19" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="19" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>31</v>
       </c>
@@ -1982,10 +1982,10 @@
         <v>140</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G19" s="11" t="s">
         <v>143</v>
@@ -2015,7 +2015,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="20" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="20" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>31</v>
       </c>
@@ -2029,10 +2029,10 @@
         <v>140</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G20" s="11" t="s">
         <v>143</v>
@@ -2060,7 +2060,7 @@
       </c>
       <c r="Q20" s="12"/>
     </row>
-    <row r="21" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="21" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>31</v>
       </c>
@@ -2074,10 +2074,10 @@
         <v>140</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G21" s="11" t="s">
         <v>143</v>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="Q21" s="12"/>
     </row>
-    <row r="22" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="22" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>31</v>
       </c>
@@ -2119,10 +2119,10 @@
         <v>140</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="G22" s="11" t="s">
         <v>143</v>
@@ -2152,33 +2152,33 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="23" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H23" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J23" s="11"/>
       <c r="K23" s="11"/>
@@ -2197,33 +2197,33 @@
       </c>
       <c r="Q23" s="12"/>
     </row>
-    <row r="24" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="24" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E24" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H24" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J24" s="11"/>
       <c r="K24" s="11"/>
@@ -2242,33 +2242,33 @@
       </c>
       <c r="Q24" s="12"/>
     </row>
-    <row r="25" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="25" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E25" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H25" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J25" s="11"/>
       <c r="K25" s="11"/>
@@ -2287,33 +2287,33 @@
       </c>
       <c r="Q25" s="12"/>
     </row>
-    <row r="26" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="26" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E26" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H26" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J26" s="11"/>
       <c r="K26" s="11"/>
@@ -2332,33 +2332,33 @@
       </c>
       <c r="Q26" s="12"/>
     </row>
-    <row r="27" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="27" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E27" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H27" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J27" s="11"/>
       <c r="K27" s="11"/>
@@ -2379,33 +2379,33 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="28" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E28" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H28" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J28" s="11"/>
       <c r="K28" s="11"/>
@@ -2424,33 +2424,33 @@
       </c>
       <c r="Q28" s="12"/>
     </row>
-    <row r="29" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="29" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E29" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H29" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J29" s="11"/>
       <c r="K29" s="11"/>
@@ -2471,33 +2471,33 @@
         <v>119</v>
       </c>
     </row>
-    <row r="30" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="30" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E30" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H30" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J30" s="11"/>
       <c r="K30" s="11"/>
@@ -2516,33 +2516,33 @@
       </c>
       <c r="Q30" s="12"/>
     </row>
-    <row r="31" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="31" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E31" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H31" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J31" s="11"/>
       <c r="K31" s="11"/>
@@ -2561,33 +2561,33 @@
       </c>
       <c r="Q31" s="12"/>
     </row>
-    <row r="32" spans="1:17" s="15" customFormat="1" ht="28.7">
+    <row r="32" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E32" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H32" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J32" s="11"/>
       <c r="K32" s="11"/>
@@ -2608,31 +2608,31 @@
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:17" s="15" customFormat="1">
+    <row r="33" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C33" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E33" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D33" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E33" s="13" t="s">
+      <c r="F33" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="F33" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="G33" s="11"/>
       <c r="H33" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J33" s="11"/>
       <c r="K33" s="11"/>
@@ -2651,31 +2651,31 @@
       </c>
       <c r="Q33" s="12"/>
     </row>
-    <row r="34" spans="1:17" s="15" customFormat="1">
+    <row r="34" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C34" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E34" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D34" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E34" s="13" t="s">
+      <c r="F34" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="F34" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="G34" s="11"/>
       <c r="H34" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J34" s="11"/>
       <c r="K34" s="11"/>
@@ -2694,31 +2694,31 @@
       </c>
       <c r="Q34" s="12"/>
     </row>
-    <row r="35" spans="1:17" s="15" customFormat="1">
+    <row r="35" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C35" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E35" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D35" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E35" s="13" t="s">
+      <c r="F35" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="F35" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="G35" s="11"/>
       <c r="H35" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J35" s="11"/>
       <c r="K35" s="11"/>
@@ -2737,31 +2737,31 @@
       </c>
       <c r="Q35" s="12"/>
     </row>
-    <row r="36" spans="1:17" s="15" customFormat="1">
+    <row r="36" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C36" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E36" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D36" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E36" s="13" t="s">
+      <c r="F36" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="F36" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="G36" s="11"/>
       <c r="H36" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J36" s="11"/>
       <c r="K36" s="11"/>
@@ -2780,31 +2780,31 @@
       </c>
       <c r="Q36" s="12"/>
     </row>
-    <row r="37" spans="1:17" s="15" customFormat="1">
+    <row r="37" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C37" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E37" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D37" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E37" s="13" t="s">
+      <c r="F37" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="F37" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="G37" s="11"/>
       <c r="H37" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J37" s="11"/>
       <c r="K37" s="11"/>
@@ -2825,31 +2825,31 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:17" s="15" customFormat="1">
+    <row r="38" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C38" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E38" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D38" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E38" s="13" t="s">
+      <c r="F38" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="G38" s="11"/>
       <c r="H38" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J38" s="11"/>
       <c r="K38" s="11"/>
@@ -2868,31 +2868,31 @@
       </c>
       <c r="Q38" s="12"/>
     </row>
-    <row r="39" spans="1:17" s="15" customFormat="1">
+    <row r="39" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C39" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E39" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D39" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E39" s="13" t="s">
+      <c r="F39" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="F39" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="G39" s="11"/>
       <c r="H39" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J39" s="11"/>
       <c r="K39" s="11"/>
@@ -2913,31 +2913,31 @@
         <v>119</v>
       </c>
     </row>
-    <row r="40" spans="1:17" s="15" customFormat="1">
+    <row r="40" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C40" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E40" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D40" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E40" s="13" t="s">
+      <c r="F40" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="F40" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="G40" s="11"/>
       <c r="H40" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J40" s="11"/>
       <c r="K40" s="11"/>
@@ -2956,31 +2956,31 @@
       </c>
       <c r="Q40" s="12"/>
     </row>
-    <row r="41" spans="1:17" s="15" customFormat="1">
+    <row r="41" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C41" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E41" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D41" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E41" s="13" t="s">
+      <c r="F41" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="F41" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="G41" s="11"/>
       <c r="H41" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J41" s="11"/>
       <c r="K41" s="11"/>
@@ -2999,31 +2999,31 @@
       </c>
       <c r="Q41" s="12"/>
     </row>
-    <row r="42" spans="1:17" s="15" customFormat="1">
+    <row r="42" spans="1:17" s="15" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C42" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E42" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D42" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E42" s="13" t="s">
+      <c r="F42" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="F42" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="G42" s="11"/>
       <c r="H42" s="11" t="s">
         <v>18</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J42" s="11"/>
       <c r="K42" s="11"/>
@@ -3137,25 +3137,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D118C320-5B2C-4B05-837B-4243603672BC}">
   <dimension ref="A1:AG99"/>
-  <sheetFormatPr defaultRowHeight="14.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="4" width="9" style="10"/>
-    <col min="6" max="6" width="12.87890625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.29296875" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.28515625" customWidth="1"/>
     <col min="8" max="8" width="32" customWidth="1"/>
-    <col min="9" max="9" width="10.87890625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.1171875" customWidth="1"/>
-    <col min="13" max="13" width="9.703125" customWidth="1"/>
-    <col min="15" max="15" width="52.87890625" customWidth="1"/>
-    <col min="16" max="16" width="12.703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="23.29296875" customWidth="1"/>
-    <col min="19" max="19" width="9.5859375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="30.29296875" customWidth="1"/>
-    <col min="21" max="21" width="21.29296875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.41015625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" customWidth="1"/>
+    <col min="13" max="13" width="9.7109375" customWidth="1"/>
+    <col min="15" max="15" width="52.85546875" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23.28515625" customWidth="1"/>
+    <col min="19" max="19" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="30.28515625" customWidth="1"/>
+    <col min="21" max="21" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="37.700000000000003">
+    <row r="1" spans="1:33" ht="39" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -3253,7 +3253,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:33" s="14" customFormat="1" ht="37">
+    <row r="2" spans="1:33" s="14" customFormat="1" ht="39" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>31</v>
       </c>
@@ -3289,7 +3289,7 @@
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
       <c r="O2" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
@@ -3331,7 +3331,7 @@
       <c r="AE2" s="4"/>
       <c r="AF2" s="4"/>
     </row>
-    <row r="3" spans="1:33" s="14" customFormat="1" ht="37">
+    <row r="3" spans="1:33" s="14" customFormat="1" ht="39" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>31</v>
       </c>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="N3" s="4"/>
       <c r="O3" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
@@ -3413,7 +3413,7 @@
       <c r="AE3" s="4"/>
       <c r="AF3" s="4"/>
     </row>
-    <row r="4" spans="1:33" s="14" customFormat="1">
+    <row r="4" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>31</v>
       </c>
@@ -3481,7 +3481,7 @@
       <c r="AE4" s="4"/>
       <c r="AF4" s="4"/>
     </row>
-    <row r="5" spans="1:33" s="14" customFormat="1">
+    <row r="5" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>31</v>
       </c>
@@ -3549,7 +3549,7 @@
       <c r="AE5" s="4"/>
       <c r="AF5" s="4"/>
     </row>
-    <row r="6" spans="1:33" s="14" customFormat="1" ht="25">
+    <row r="6" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>31</v>
       </c>
@@ -3629,7 +3629,7 @@
       <c r="AE6" s="4"/>
       <c r="AF6" s="4"/>
     </row>
-    <row r="7" spans="1:33" s="14" customFormat="1">
+    <row r="7" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
@@ -3709,7 +3709,7 @@
       <c r="AE7" s="4"/>
       <c r="AF7" s="4"/>
     </row>
-    <row r="8" spans="1:33" s="14" customFormat="1" ht="25">
+    <row r="8" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>31</v>
       </c>
@@ -3787,7 +3787,7 @@
       <c r="AE8" s="4"/>
       <c r="AF8" s="4"/>
     </row>
-    <row r="9" spans="1:33" s="14" customFormat="1" ht="25">
+    <row r="9" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>31</v>
       </c>
@@ -3869,7 +3869,7 @@
       <c r="AE9" s="4"/>
       <c r="AF9" s="4"/>
     </row>
-    <row r="10" spans="1:33" s="14" customFormat="1" ht="25">
+    <row r="10" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>31</v>
       </c>
@@ -3951,7 +3951,7 @@
       <c r="AE10" s="4"/>
       <c r="AF10" s="4"/>
     </row>
-    <row r="11" spans="1:33" s="14" customFormat="1" ht="25">
+    <row r="11" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>31</v>
       </c>
@@ -4031,7 +4031,7 @@
       <c r="AE11" s="4"/>
       <c r="AF11" s="4"/>
     </row>
-    <row r="12" spans="1:33" s="14" customFormat="1">
+    <row r="12" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>31</v>
       </c>
@@ -4105,7 +4105,7 @@
       <c r="AE12" s="4"/>
       <c r="AF12" s="4"/>
     </row>
-    <row r="13" spans="1:33" s="14" customFormat="1">
+    <row r="13" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>31</v>
       </c>
@@ -4179,12 +4179,12 @@
       <c r="AE13" s="4"/>
       <c r="AF13" s="4"/>
     </row>
-    <row r="14" spans="1:33" s="14" customFormat="1">
+    <row r="14" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>130</v>
@@ -4197,10 +4197,10 @@
         <v>92</v>
       </c>
       <c r="G14" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H14" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="H14" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="I14" s="11" t="s">
         <v>93</v>
@@ -4255,15 +4255,15 @@
       <c r="AE14" s="11"/>
       <c r="AF14" s="11"/>
       <c r="AG14" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
-    <row r="15" spans="1:33" s="14" customFormat="1" ht="28.7">
+    <row r="15" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>130</v>
@@ -4276,10 +4276,10 @@
         <v>92</v>
       </c>
       <c r="G15" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H15" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="H15" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="I15" s="11" t="s">
         <v>95</v>
@@ -4299,10 +4299,10 @@
       <c r="N15" s="11"/>
       <c r="O15" s="12"/>
       <c r="P15" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="Q15" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="R15" s="11" t="s">
         <v>41</v>
@@ -4342,12 +4342,12 @@
       <c r="AE15" s="11"/>
       <c r="AF15" s="11"/>
     </row>
-    <row r="16" spans="1:33" s="14" customFormat="1">
+    <row r="16" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>130</v>
@@ -4360,10 +4360,10 @@
         <v>92</v>
       </c>
       <c r="G16" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H16" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="I16" s="11" t="s">
         <v>99</v>
@@ -4410,12 +4410,12 @@
       <c r="AE16" s="11"/>
       <c r="AF16" s="11"/>
     </row>
-    <row r="17" spans="1:32" s="14" customFormat="1">
+    <row r="17" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>130</v>
@@ -4428,10 +4428,10 @@
         <v>92</v>
       </c>
       <c r="G17" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H17" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="H17" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="I17" s="11" t="s">
         <v>100</v>
@@ -4478,12 +4478,12 @@
       <c r="AE17" s="11"/>
       <c r="AF17" s="11"/>
     </row>
-    <row r="18" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="18" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>130</v>
@@ -4496,10 +4496,10 @@
         <v>92</v>
       </c>
       <c r="G18" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H18" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="H18" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="I18" s="11" t="s">
         <v>101</v>
@@ -4562,12 +4562,12 @@
       <c r="AE18" s="11"/>
       <c r="AF18" s="11"/>
     </row>
-    <row r="19" spans="1:32" s="14" customFormat="1">
+    <row r="19" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>130</v>
@@ -4580,10 +4580,10 @@
         <v>92</v>
       </c>
       <c r="G19" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H19" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="H19" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="I19" s="11" t="s">
         <v>102</v>
@@ -4646,12 +4646,12 @@
       <c r="AE19" s="11"/>
       <c r="AF19" s="11"/>
     </row>
-    <row r="20" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="20" spans="1:32" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>130</v>
@@ -4664,10 +4664,10 @@
         <v>92</v>
       </c>
       <c r="G20" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H20" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="H20" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="I20" s="11" t="s">
         <v>106</v>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="N20" s="11"/>
       <c r="O20" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P20" s="11"/>
       <c r="Q20" s="11"/>
@@ -4728,12 +4728,12 @@
       <c r="AE20" s="11"/>
       <c r="AF20" s="11"/>
     </row>
-    <row r="21" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="21" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>130</v>
@@ -4746,10 +4746,10 @@
         <v>92</v>
       </c>
       <c r="G21" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H21" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="H21" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="I21" s="4" t="s">
         <v>124</v>
@@ -4810,12 +4810,12 @@
       <c r="AE21" s="4"/>
       <c r="AF21" s="4"/>
     </row>
-    <row r="22" spans="1:32" s="14" customFormat="1">
+    <row r="22" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>130</v>
@@ -4828,10 +4828,10 @@
         <v>92</v>
       </c>
       <c r="G22" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H22" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="I22" s="11" t="s">
         <v>109</v>
@@ -4884,12 +4884,12 @@
       <c r="AE22" s="11"/>
       <c r="AF22" s="11"/>
     </row>
-    <row r="23" spans="1:32" s="14" customFormat="1">
+    <row r="23" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>130</v>
@@ -4902,10 +4902,10 @@
         <v>92</v>
       </c>
       <c r="G23" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H23" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="H23" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="I23" s="11" t="s">
         <v>111</v>
@@ -4958,7 +4958,7 @@
       <c r="AE23" s="11"/>
       <c r="AF23" s="11"/>
     </row>
-    <row r="24" spans="1:32" s="14" customFormat="1">
+    <row r="24" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>31</v>
       </c>
@@ -5034,7 +5034,7 @@
       <c r="AE24" s="4"/>
       <c r="AF24" s="4"/>
     </row>
-    <row r="25" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="25" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>31</v>
       </c>
@@ -5076,7 +5076,7 @@
       <c r="O25" s="5"/>
       <c r="P25" s="4"/>
       <c r="Q25" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="R25" s="4" t="s">
         <v>41</v>
@@ -5116,7 +5116,7 @@
       <c r="AE25" s="4"/>
       <c r="AF25" s="4"/>
     </row>
-    <row r="26" spans="1:32" s="14" customFormat="1">
+    <row r="26" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>31</v>
       </c>
@@ -5184,7 +5184,7 @@
       <c r="AE26" s="4"/>
       <c r="AF26" s="4"/>
     </row>
-    <row r="27" spans="1:32" s="14" customFormat="1">
+    <row r="27" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>31</v>
       </c>
@@ -5252,7 +5252,7 @@
       <c r="AE27" s="4"/>
       <c r="AF27" s="4"/>
     </row>
-    <row r="28" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="28" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>31</v>
       </c>
@@ -5336,7 +5336,7 @@
       <c r="AE28" s="4"/>
       <c r="AF28" s="4"/>
     </row>
-    <row r="29" spans="1:32" s="14" customFormat="1">
+    <row r="29" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>31</v>
       </c>
@@ -5420,7 +5420,7 @@
       <c r="AE29" s="4"/>
       <c r="AF29" s="4"/>
     </row>
-    <row r="30" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="30" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>31</v>
       </c>
@@ -5500,7 +5500,7 @@
       <c r="AE30" s="4"/>
       <c r="AF30" s="4"/>
     </row>
-    <row r="31" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="31" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>31</v>
       </c>
@@ -5582,7 +5582,7 @@
       <c r="AE31" s="4"/>
       <c r="AF31" s="4"/>
     </row>
-    <row r="32" spans="1:32" s="14" customFormat="1">
+    <row r="32" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>31</v>
       </c>
@@ -5656,7 +5656,7 @@
       <c r="AE32" s="4"/>
       <c r="AF32" s="4"/>
     </row>
-    <row r="33" spans="1:32" s="14" customFormat="1">
+    <row r="33" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>31</v>
       </c>
@@ -5730,12 +5730,12 @@
       <c r="AE33" s="4"/>
       <c r="AF33" s="4"/>
     </row>
-    <row r="34" spans="1:32" s="14" customFormat="1">
+    <row r="34" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>32</v>
@@ -5748,10 +5748,10 @@
         <v>92</v>
       </c>
       <c r="G34" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H34" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="H34" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="I34" s="4" t="s">
         <v>93</v>
@@ -5806,12 +5806,12 @@
       <c r="AE34" s="4"/>
       <c r="AF34" s="4"/>
     </row>
-    <row r="35" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="35" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>32</v>
@@ -5824,10 +5824,10 @@
         <v>92</v>
       </c>
       <c r="G35" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H35" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="H35" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="I35" s="4" t="s">
         <v>95</v>
@@ -5847,10 +5847,10 @@
       <c r="N35" s="4"/>
       <c r="O35" s="5"/>
       <c r="P35" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="Q35" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R35" s="4" t="s">
         <v>41</v>
@@ -5890,12 +5890,12 @@
       <c r="AE35" s="4"/>
       <c r="AF35" s="4"/>
     </row>
-    <row r="36" spans="1:32" s="14" customFormat="1">
+    <row r="36" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>32</v>
@@ -5908,10 +5908,10 @@
         <v>92</v>
       </c>
       <c r="G36" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H36" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="H36" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="I36" s="4" t="s">
         <v>99</v>
@@ -5958,12 +5958,12 @@
       <c r="AE36" s="4"/>
       <c r="AF36" s="4"/>
     </row>
-    <row r="37" spans="1:32" s="14" customFormat="1">
+    <row r="37" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>32</v>
@@ -5976,10 +5976,10 @@
         <v>92</v>
       </c>
       <c r="G37" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H37" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="H37" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="I37" s="4" t="s">
         <v>100</v>
@@ -6026,12 +6026,12 @@
       <c r="AE37" s="4"/>
       <c r="AF37" s="4"/>
     </row>
-    <row r="38" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="38" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>32</v>
@@ -6044,10 +6044,10 @@
         <v>92</v>
       </c>
       <c r="G38" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H38" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="H38" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="I38" s="4" t="s">
         <v>101</v>
@@ -6110,12 +6110,12 @@
       <c r="AE38" s="4"/>
       <c r="AF38" s="4"/>
     </row>
-    <row r="39" spans="1:32" s="14" customFormat="1">
+    <row r="39" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>32</v>
@@ -6128,10 +6128,10 @@
         <v>92</v>
       </c>
       <c r="G39" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H39" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="H39" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="I39" s="4" t="s">
         <v>102</v>
@@ -6194,12 +6194,12 @@
       <c r="AE39" s="4"/>
       <c r="AF39" s="4"/>
     </row>
-    <row r="40" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="40" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>32</v>
@@ -6212,10 +6212,10 @@
         <v>92</v>
       </c>
       <c r="G40" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H40" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="H40" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="I40" s="4" t="s">
         <v>106</v>
@@ -6274,12 +6274,12 @@
       <c r="AE40" s="4"/>
       <c r="AF40" s="4"/>
     </row>
-    <row r="41" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="41" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>32</v>
@@ -6292,10 +6292,10 @@
         <v>92</v>
       </c>
       <c r="G41" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H41" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="H41" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="I41" s="4" t="s">
         <v>124</v>
@@ -6356,12 +6356,12 @@
       <c r="AE41" s="4"/>
       <c r="AF41" s="4"/>
     </row>
-    <row r="42" spans="1:32" s="14" customFormat="1">
+    <row r="42" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C42" s="11" t="s">
         <v>32</v>
@@ -6374,10 +6374,10 @@
         <v>92</v>
       </c>
       <c r="G42" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H42" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="H42" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="I42" s="4" t="s">
         <v>109</v>
@@ -6430,12 +6430,12 @@
       <c r="AE42" s="4"/>
       <c r="AF42" s="4"/>
     </row>
-    <row r="43" spans="1:32" s="14" customFormat="1">
+    <row r="43" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>32</v>
@@ -6448,10 +6448,10 @@
         <v>92</v>
       </c>
       <c r="G43" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H43" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="H43" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="I43" s="4" t="s">
         <v>111</v>
@@ -6504,12 +6504,12 @@
       <c r="AE43" s="4"/>
       <c r="AF43" s="4"/>
     </row>
-    <row r="44" spans="1:32" s="14" customFormat="1">
+    <row r="44" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C44" s="11" t="s">
         <v>32</v>
@@ -6522,10 +6522,10 @@
         <v>92</v>
       </c>
       <c r="G44" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I44" s="4" t="s">
         <v>93</v>
@@ -6580,12 +6580,12 @@
       <c r="AE44" s="4"/>
       <c r="AF44" s="4"/>
     </row>
-    <row r="45" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="45" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C45" s="11" t="s">
         <v>32</v>
@@ -6598,10 +6598,10 @@
         <v>92</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I45" s="4" t="s">
         <v>95</v>
@@ -6621,10 +6621,10 @@
       <c r="N45" s="4"/>
       <c r="O45" s="5"/>
       <c r="P45" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Q45" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R45" s="4" t="s">
         <v>41</v>
@@ -6664,12 +6664,12 @@
       <c r="AE45" s="4"/>
       <c r="AF45" s="4"/>
     </row>
-    <row r="46" spans="1:32" s="14" customFormat="1">
+    <row r="46" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C46" s="11" t="s">
         <v>32</v>
@@ -6682,10 +6682,10 @@
         <v>92</v>
       </c>
       <c r="G46" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H46" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I46" s="4" t="s">
         <v>99</v>
@@ -6732,12 +6732,12 @@
       <c r="AE46" s="4"/>
       <c r="AF46" s="4"/>
     </row>
-    <row r="47" spans="1:32" s="14" customFormat="1">
+    <row r="47" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C47" s="11" t="s">
         <v>32</v>
@@ -6750,10 +6750,10 @@
         <v>92</v>
       </c>
       <c r="G47" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H47" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I47" s="4" t="s">
         <v>100</v>
@@ -6800,12 +6800,12 @@
       <c r="AE47" s="4"/>
       <c r="AF47" s="4"/>
     </row>
-    <row r="48" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="48" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C48" s="11" t="s">
         <v>32</v>
@@ -6818,10 +6818,10 @@
         <v>92</v>
       </c>
       <c r="G48" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H48" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I48" s="4" t="s">
         <v>101</v>
@@ -6884,12 +6884,12 @@
       <c r="AE48" s="4"/>
       <c r="AF48" s="4"/>
     </row>
-    <row r="49" spans="1:32" s="14" customFormat="1">
+    <row r="49" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C49" s="11" t="s">
         <v>32</v>
@@ -6902,10 +6902,10 @@
         <v>92</v>
       </c>
       <c r="G49" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H49" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>102</v>
@@ -6968,12 +6968,12 @@
       <c r="AE49" s="4"/>
       <c r="AF49" s="4"/>
     </row>
-    <row r="50" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="50" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C50" s="11" t="s">
         <v>32</v>
@@ -6986,10 +6986,10 @@
         <v>92</v>
       </c>
       <c r="G50" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H50" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I50" s="4" t="s">
         <v>106</v>
@@ -7048,12 +7048,12 @@
       <c r="AE50" s="4"/>
       <c r="AF50" s="4"/>
     </row>
-    <row r="51" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="51" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C51" s="11" t="s">
         <v>32</v>
@@ -7066,10 +7066,10 @@
         <v>92</v>
       </c>
       <c r="G51" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H51" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>124</v>
@@ -7130,12 +7130,12 @@
       <c r="AE51" s="4"/>
       <c r="AF51" s="4"/>
     </row>
-    <row r="52" spans="1:32" s="14" customFormat="1">
+    <row r="52" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C52" s="11" t="s">
         <v>32</v>
@@ -7148,10 +7148,10 @@
         <v>92</v>
       </c>
       <c r="G52" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>109</v>
@@ -7204,12 +7204,12 @@
       <c r="AE52" s="4"/>
       <c r="AF52" s="4"/>
     </row>
-    <row r="53" spans="1:32" s="14" customFormat="1">
+    <row r="53" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C53" s="11" t="s">
         <v>32</v>
@@ -7222,10 +7222,10 @@
         <v>92</v>
       </c>
       <c r="G53" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H53" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>111</v>
@@ -7278,7 +7278,7 @@
       <c r="AE53" s="4"/>
       <c r="AF53" s="4"/>
     </row>
-    <row r="54" spans="1:32" s="14" customFormat="1">
+    <row r="54" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
         <v>31</v>
       </c>
@@ -7296,10 +7296,10 @@
         <v>92</v>
       </c>
       <c r="G54" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H54" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I54" s="11" t="s">
         <v>93</v>
@@ -7354,7 +7354,7 @@
       <c r="AE54" s="11"/>
       <c r="AF54" s="11"/>
     </row>
-    <row r="55" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="55" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
         <v>31</v>
       </c>
@@ -7372,10 +7372,10 @@
         <v>92</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H55" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I55" s="11" t="s">
         <v>95</v>
@@ -7398,7 +7398,7 @@
         <v>140</v>
       </c>
       <c r="Q55" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R55" s="11" t="s">
         <v>41</v>
@@ -7438,7 +7438,7 @@
       <c r="AE55" s="11"/>
       <c r="AF55" s="11"/>
     </row>
-    <row r="56" spans="1:32" s="14" customFormat="1">
+    <row r="56" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
         <v>31</v>
       </c>
@@ -7456,10 +7456,10 @@
         <v>92</v>
       </c>
       <c r="G56" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H56" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I56" s="11" t="s">
         <v>99</v>
@@ -7506,7 +7506,7 @@
       <c r="AE56" s="11"/>
       <c r="AF56" s="11"/>
     </row>
-    <row r="57" spans="1:32" s="14" customFormat="1">
+    <row r="57" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
         <v>31</v>
       </c>
@@ -7524,10 +7524,10 @@
         <v>92</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H57" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I57" s="11" t="s">
         <v>100</v>
@@ -7574,7 +7574,7 @@
       <c r="AE57" s="11"/>
       <c r="AF57" s="11"/>
     </row>
-    <row r="58" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="58" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
         <v>31</v>
       </c>
@@ -7592,10 +7592,10 @@
         <v>92</v>
       </c>
       <c r="G58" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H58" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I58" s="11" t="s">
         <v>101</v>
@@ -7658,7 +7658,7 @@
       <c r="AE58" s="11"/>
       <c r="AF58" s="11"/>
     </row>
-    <row r="59" spans="1:32" s="14" customFormat="1">
+    <row r="59" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
         <v>31</v>
       </c>
@@ -7676,10 +7676,10 @@
         <v>92</v>
       </c>
       <c r="G59" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H59" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I59" s="11" t="s">
         <v>102</v>
@@ -7742,7 +7742,7 @@
       <c r="AE59" s="11"/>
       <c r="AF59" s="11"/>
     </row>
-    <row r="60" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="60" spans="1:32" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
         <v>31</v>
       </c>
@@ -7760,10 +7760,10 @@
         <v>92</v>
       </c>
       <c r="G60" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H60" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I60" s="11" t="s">
         <v>106</v>
@@ -7783,10 +7783,10 @@
       <c r="N60" s="11"/>
       <c r="O60" s="12"/>
       <c r="P60" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="Q60" s="11" t="s">
         <v>171</v>
-      </c>
-      <c r="Q60" s="11" t="s">
-        <v>172</v>
       </c>
       <c r="R60" s="11" t="s">
         <v>41</v>
@@ -7826,7 +7826,7 @@
       <c r="AE60" s="11"/>
       <c r="AF60" s="11"/>
     </row>
-    <row r="61" spans="1:32" s="14" customFormat="1">
+    <row r="61" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
         <v>31</v>
       </c>
@@ -7844,10 +7844,10 @@
         <v>92</v>
       </c>
       <c r="G61" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H61" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I61" s="11" t="s">
         <v>109</v>
@@ -7900,7 +7900,7 @@
       <c r="AE61" s="11"/>
       <c r="AF61" s="11"/>
     </row>
-    <row r="62" spans="1:32" s="14" customFormat="1">
+    <row r="62" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
         <v>31</v>
       </c>
@@ -7918,10 +7918,10 @@
         <v>92</v>
       </c>
       <c r="G62" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H62" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I62" s="11" t="s">
         <v>111</v>
@@ -7974,7 +7974,7 @@
       <c r="AE62" s="11"/>
       <c r="AF62" s="11"/>
     </row>
-    <row r="63" spans="1:32" s="14" customFormat="1">
+    <row r="63" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
         <v>31</v>
       </c>
@@ -7992,10 +7992,10 @@
         <v>92</v>
       </c>
       <c r="G63" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H63" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I63" s="11" t="s">
         <v>93</v>
@@ -8050,7 +8050,7 @@
       <c r="AE63" s="11"/>
       <c r="AF63" s="11"/>
     </row>
-    <row r="64" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="64" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
         <v>31</v>
       </c>
@@ -8068,10 +8068,10 @@
         <v>92</v>
       </c>
       <c r="G64" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H64" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I64" s="11" t="s">
         <v>95</v>
@@ -8094,7 +8094,7 @@
         <v>140</v>
       </c>
       <c r="Q64" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R64" s="11" t="s">
         <v>41</v>
@@ -8134,7 +8134,7 @@
       <c r="AE64" s="11"/>
       <c r="AF64" s="11"/>
     </row>
-    <row r="65" spans="1:32" s="14" customFormat="1">
+    <row r="65" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
         <v>31</v>
       </c>
@@ -8152,10 +8152,10 @@
         <v>92</v>
       </c>
       <c r="G65" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H65" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I65" s="11" t="s">
         <v>99</v>
@@ -8202,7 +8202,7 @@
       <c r="AE65" s="11"/>
       <c r="AF65" s="11"/>
     </row>
-    <row r="66" spans="1:32" s="14" customFormat="1">
+    <row r="66" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
         <v>31</v>
       </c>
@@ -8220,10 +8220,10 @@
         <v>92</v>
       </c>
       <c r="G66" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I66" s="11" t="s">
         <v>100</v>
@@ -8270,7 +8270,7 @@
       <c r="AE66" s="11"/>
       <c r="AF66" s="11"/>
     </row>
-    <row r="67" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="67" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
         <v>31</v>
       </c>
@@ -8288,10 +8288,10 @@
         <v>92</v>
       </c>
       <c r="G67" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H67" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I67" s="11" t="s">
         <v>101</v>
@@ -8354,7 +8354,7 @@
       <c r="AE67" s="11"/>
       <c r="AF67" s="11"/>
     </row>
-    <row r="68" spans="1:32" s="14" customFormat="1">
+    <row r="68" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
         <v>31</v>
       </c>
@@ -8372,10 +8372,10 @@
         <v>92</v>
       </c>
       <c r="G68" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H68" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I68" s="11" t="s">
         <v>102</v>
@@ -8438,7 +8438,7 @@
       <c r="AE68" s="11"/>
       <c r="AF68" s="11"/>
     </row>
-    <row r="69" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="69" spans="1:32" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
         <v>31</v>
       </c>
@@ -8456,10 +8456,10 @@
         <v>92</v>
       </c>
       <c r="G69" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H69" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I69" s="11" t="s">
         <v>106</v>
@@ -8479,10 +8479,10 @@
       <c r="N69" s="11"/>
       <c r="O69" s="12"/>
       <c r="P69" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q69" s="11" t="s">
         <v>176</v>
-      </c>
-      <c r="Q69" s="11" t="s">
-        <v>177</v>
       </c>
       <c r="R69" s="11" t="s">
         <v>41</v>
@@ -8522,7 +8522,7 @@
       <c r="AE69" s="11"/>
       <c r="AF69" s="11"/>
     </row>
-    <row r="70" spans="1:32" s="14" customFormat="1">
+    <row r="70" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
         <v>31</v>
       </c>
@@ -8540,10 +8540,10 @@
         <v>92</v>
       </c>
       <c r="G70" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H70" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I70" s="11" t="s">
         <v>109</v>
@@ -8596,7 +8596,7 @@
       <c r="AE70" s="11"/>
       <c r="AF70" s="11"/>
     </row>
-    <row r="71" spans="1:32" s="14" customFormat="1">
+    <row r="71" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
         <v>31</v>
       </c>
@@ -8614,10 +8614,10 @@
         <v>92</v>
       </c>
       <c r="G71" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H71" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I71" s="11" t="s">
         <v>111</v>
@@ -8670,7 +8670,7 @@
       <c r="AE71" s="11"/>
       <c r="AF71" s="11"/>
     </row>
-    <row r="72" spans="1:32" s="14" customFormat="1">
+    <row r="72" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
         <v>31</v>
       </c>
@@ -8688,10 +8688,10 @@
         <v>92</v>
       </c>
       <c r="G72" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H72" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I72" s="11" t="s">
         <v>93</v>
@@ -8746,7 +8746,7 @@
       <c r="AE72" s="11"/>
       <c r="AF72" s="11"/>
     </row>
-    <row r="73" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="73" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
         <v>31</v>
       </c>
@@ -8764,10 +8764,10 @@
         <v>92</v>
       </c>
       <c r="G73" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H73" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I73" s="11" t="s">
         <v>95</v>
@@ -8790,7 +8790,7 @@
         <v>140</v>
       </c>
       <c r="Q73" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="R73" s="11" t="s">
         <v>41</v>
@@ -8830,7 +8830,7 @@
       <c r="AE73" s="11"/>
       <c r="AF73" s="11"/>
     </row>
-    <row r="74" spans="1:32" s="14" customFormat="1">
+    <row r="74" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
         <v>31</v>
       </c>
@@ -8848,10 +8848,10 @@
         <v>92</v>
       </c>
       <c r="G74" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H74" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I74" s="11" t="s">
         <v>99</v>
@@ -8898,7 +8898,7 @@
       <c r="AE74" s="11"/>
       <c r="AF74" s="11"/>
     </row>
-    <row r="75" spans="1:32" s="14" customFormat="1">
+    <row r="75" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
         <v>31</v>
       </c>
@@ -8916,10 +8916,10 @@
         <v>92</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H75" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I75" s="11" t="s">
         <v>100</v>
@@ -8966,7 +8966,7 @@
       <c r="AE75" s="11"/>
       <c r="AF75" s="11"/>
     </row>
-    <row r="76" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="76" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
         <v>31</v>
       </c>
@@ -8984,10 +8984,10 @@
         <v>92</v>
       </c>
       <c r="G76" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H76" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I76" s="11" t="s">
         <v>101</v>
@@ -9050,7 +9050,7 @@
       <c r="AE76" s="11"/>
       <c r="AF76" s="11"/>
     </row>
-    <row r="77" spans="1:32" s="14" customFormat="1">
+    <row r="77" spans="1:32" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
         <v>31</v>
       </c>
@@ -9068,10 +9068,10 @@
         <v>92</v>
       </c>
       <c r="G77" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H77" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I77" s="11" t="s">
         <v>102</v>
@@ -9134,7 +9134,7 @@
       <c r="AE77" s="11"/>
       <c r="AF77" s="11"/>
     </row>
-    <row r="78" spans="1:32" s="14" customFormat="1" ht="28.7">
+    <row r="78" spans="1:32" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
         <v>31</v>
       </c>
@@ -9152,10 +9152,10 @@
         <v>92</v>
       </c>
       <c r="G78" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H78" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I78" s="11" t="s">
         <v>106</v>
@@ -9175,10 +9175,10 @@
       <c r="N78" s="11"/>
       <c r="O78" s="12"/>
       <c r="P78" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q78" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="R78" s="11" t="s">
         <v>41</v>
@@ -9218,7 +9218,7 @@
       <c r="AE78" s="11"/>
       <c r="AF78" s="11"/>
     </row>
-    <row r="79" spans="1:32" s="14" customFormat="1">
+    <row r="79" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
         <v>31</v>
       </c>
@@ -9236,10 +9236,10 @@
         <v>92</v>
       </c>
       <c r="G79" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H79" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I79" s="11" t="s">
         <v>109</v>
@@ -9292,7 +9292,7 @@
       <c r="AE79" s="11"/>
       <c r="AF79" s="11"/>
     </row>
-    <row r="80" spans="1:32" s="14" customFormat="1">
+    <row r="80" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
         <v>31</v>
       </c>
@@ -9310,10 +9310,10 @@
         <v>92</v>
       </c>
       <c r="G80" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H80" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I80" s="11" t="s">
         <v>111</v>
@@ -9366,12 +9366,12 @@
       <c r="AE80" s="11"/>
       <c r="AF80" s="11"/>
     </row>
-    <row r="81" spans="1:33" s="14" customFormat="1">
+    <row r="81" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C81" s="11" t="s">
         <v>32</v>
@@ -9384,10 +9384,10 @@
         <v>92</v>
       </c>
       <c r="G81" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="H81" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="H81" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="I81" s="4" t="s">
         <v>93</v>
@@ -9442,12 +9442,12 @@
       <c r="AE81" s="4"/>
       <c r="AF81" s="4"/>
     </row>
-    <row r="82" spans="1:33" s="14" customFormat="1" ht="25">
+    <row r="82" spans="1:33" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C82" s="11" t="s">
         <v>32</v>
@@ -9460,10 +9460,10 @@
         <v>92</v>
       </c>
       <c r="G82" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="H82" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="H82" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="I82" s="4" t="s">
         <v>95</v>
@@ -9483,10 +9483,10 @@
       <c r="N82" s="4"/>
       <c r="O82" s="5"/>
       <c r="P82" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="Q82" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R82" s="4" t="s">
         <v>41</v>
@@ -9526,12 +9526,12 @@
       <c r="AE82" s="4"/>
       <c r="AF82" s="4"/>
     </row>
-    <row r="83" spans="1:33" s="14" customFormat="1">
+    <row r="83" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C83" s="11" t="s">
         <v>32</v>
@@ -9544,10 +9544,10 @@
         <v>92</v>
       </c>
       <c r="G83" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="H83" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="H83" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>99</v>
@@ -9594,12 +9594,12 @@
       <c r="AE83" s="4"/>
       <c r="AF83" s="4"/>
     </row>
-    <row r="84" spans="1:33" s="14" customFormat="1">
+    <row r="84" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C84" s="11" t="s">
         <v>32</v>
@@ -9612,10 +9612,10 @@
         <v>92</v>
       </c>
       <c r="G84" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="H84" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="H84" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="I84" s="4" t="s">
         <v>100</v>
@@ -9662,12 +9662,12 @@
       <c r="AE84" s="4"/>
       <c r="AF84" s="4"/>
     </row>
-    <row r="85" spans="1:33" s="14" customFormat="1" ht="25">
+    <row r="85" spans="1:33" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C85" s="11" t="s">
         <v>32</v>
@@ -9680,10 +9680,10 @@
         <v>92</v>
       </c>
       <c r="G85" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="H85" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="H85" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>101</v>
@@ -9746,12 +9746,12 @@
       <c r="AE85" s="4"/>
       <c r="AF85" s="4"/>
     </row>
-    <row r="86" spans="1:33" s="14" customFormat="1">
+    <row r="86" spans="1:33" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C86" s="11" t="s">
         <v>32</v>
@@ -9764,10 +9764,10 @@
         <v>92</v>
       </c>
       <c r="G86" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="H86" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="H86" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>102</v>
@@ -9830,12 +9830,12 @@
       <c r="AE86" s="4"/>
       <c r="AF86" s="4"/>
     </row>
-    <row r="87" spans="1:33" s="14" customFormat="1" ht="25">
+    <row r="87" spans="1:33" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C87" s="11" t="s">
         <v>32</v>
@@ -9848,10 +9848,10 @@
         <v>92</v>
       </c>
       <c r="G87" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="H87" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="H87" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="I87" s="4" t="s">
         <v>106</v>
@@ -9871,10 +9871,10 @@
       <c r="N87" s="4"/>
       <c r="O87" s="5"/>
       <c r="P87" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Q87" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="R87" s="4" t="s">
         <v>41</v>
@@ -9914,12 +9914,12 @@
       <c r="AE87" s="4"/>
       <c r="AF87" s="4"/>
     </row>
-    <row r="88" spans="1:33" s="14" customFormat="1">
+    <row r="88" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C88" s="11" t="s">
         <v>32</v>
@@ -9932,10 +9932,10 @@
         <v>92</v>
       </c>
       <c r="G88" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="H88" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="H88" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="I88" s="4" t="s">
         <v>109</v>
@@ -9988,12 +9988,12 @@
       <c r="AE88" s="4"/>
       <c r="AF88" s="4"/>
     </row>
-    <row r="89" spans="1:33" s="14" customFormat="1" ht="21" customHeight="1">
+    <row r="89" spans="1:33" s="14" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C89" s="11" t="s">
         <v>32</v>
@@ -10006,10 +10006,10 @@
         <v>92</v>
       </c>
       <c r="G89" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="H89" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="H89" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="I89" s="4" t="s">
         <v>111</v>
@@ -10062,7 +10062,7 @@
       <c r="AE89" s="4"/>
       <c r="AF89" s="4"/>
     </row>
-    <row r="90" spans="1:33" s="14" customFormat="1">
+    <row r="90" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
         <v>31</v>
       </c>
@@ -10138,10 +10138,10 @@
       <c r="AE90" s="11"/>
       <c r="AF90" s="11"/>
       <c r="AG90" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
-    <row r="91" spans="1:33" s="14" customFormat="1" ht="28.7">
+    <row r="91" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="11" t="s">
         <v>31</v>
       </c>
@@ -10225,7 +10225,7 @@
       <c r="AE91" s="11"/>
       <c r="AF91" s="11"/>
     </row>
-    <row r="92" spans="1:33" s="14" customFormat="1">
+    <row r="92" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
         <v>31</v>
       </c>
@@ -10293,7 +10293,7 @@
       <c r="AE92" s="11"/>
       <c r="AF92" s="11"/>
     </row>
-    <row r="93" spans="1:33" s="14" customFormat="1">
+    <row r="93" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
         <v>31</v>
       </c>
@@ -10361,7 +10361,7 @@
       <c r="AE93" s="11"/>
       <c r="AF93" s="11"/>
     </row>
-    <row r="94" spans="1:33" s="14" customFormat="1" ht="28.7">
+    <row r="94" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
         <v>31</v>
       </c>
@@ -10445,7 +10445,7 @@
       <c r="AE94" s="11"/>
       <c r="AF94" s="11"/>
     </row>
-    <row r="95" spans="1:33" s="14" customFormat="1">
+    <row r="95" spans="1:33" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
         <v>31</v>
       </c>
@@ -10529,7 +10529,7 @@
       <c r="AE95" s="11"/>
       <c r="AF95" s="11"/>
     </row>
-    <row r="96" spans="1:33" s="14" customFormat="1" ht="28.7">
+    <row r="96" spans="1:33" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A96" s="11" t="s">
         <v>31</v>
       </c>
@@ -10611,7 +10611,7 @@
       <c r="AE96" s="11"/>
       <c r="AF96" s="11"/>
     </row>
-    <row r="97" spans="1:32" s="14" customFormat="1" ht="25">
+    <row r="97" spans="1:32" s="14" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
         <v>31</v>
       </c>
@@ -10693,7 +10693,7 @@
       <c r="AE97" s="4"/>
       <c r="AF97" s="4"/>
     </row>
-    <row r="98" spans="1:32" s="14" customFormat="1">
+    <row r="98" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="11" t="s">
         <v>31</v>
       </c>
@@ -10767,7 +10767,7 @@
       <c r="AE98" s="11"/>
       <c r="AF98" s="11"/>
     </row>
-    <row r="99" spans="1:32" s="14" customFormat="1">
+    <row r="99" spans="1:32" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
         <v>31</v>
       </c>
@@ -16455,15 +16455,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EA3DD6FD0640724CAC6A104AA4040E53" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="866aaee467307fab2f51bbdbaaea79d8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3dc215b4-4765-4137-95ef-e24fb8216673" xmlns:ns3="2634c873-c79e-4fdd-b8bf-a33e5fa5c27f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="636a025d234e12dfc0e20f1263040641" ns2:_="" ns3:_="">
     <xsd:import namespace="3dc215b4-4765-4137-95ef-e24fb8216673"/>
@@ -16720,6 +16711,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72C26AEA-38B4-45B2-94FF-5972E3017E52}">
   <ds:schemaRefs>
@@ -16732,14 +16732,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62FA68FA-8C71-4E93-80BA-49A20AA62094}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39409D45-3830-4E57-BD4D-A5503E0F1185}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16758,6 +16750,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62FA68FA-8C71-4E93-80BA-49A20AA62094}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{078244a1-de67-4c9e-9088-986d7f110a37}" enabled="0" method="" siteId="{078244a1-de67-4c9e-9088-986d7f110a37}" removed="1"/>

</xml_diff>